<commit_message>
feat: menu 'Actualizar Datos' para cargar potencia y horas desde Excel
Nuevo menu lateral (admin) para actualizar datos de calculo desde Excel:

Backend (2 endpoints):
- POST /api/import/potencia: lee 'Nro Inventario' + 'Potencia W',
  actualiza maquinas_potencia.potencia y recalcula el consumo
- POST /api/import/horas: lee 'Nro Inventario' + 'HS/DIA', actualiza
  inventario_mensual.hs_dia del periodo seleccionado y recalcula
- Helper extraerMapeoInventario: detecta la hoja correcta por columnas
- Registro en audit log de cada actualizacion

Frontend:
- Nuevo item de menu 'Actualizar Datos'
- Dos tarjetas: subir Potencia y subir Horas (con selector de periodo)
- Zonas de carga, resultados OK/error, toasts

Verificado con archivos reales:
- Potencia: 1053/1056 maquinas actualizadas
- Horas: 845/852 maquinas actualizadas para el periodo
- Recalculo correcto (potencia x hs_dia)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RE_ Horas de uso de máquinas - pendientes/Horas de uso - relevamiento operaciones filtrado.xlsx
+++ b/RE_ Horas de uso de máquinas - pendientes/Horas de uso - relevamiento operaciones filtrado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nuevo Calculo de Consumo electrico\RE_ Horas de uso de máquinas - pendientes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60DBB923-BE08-4822-B9C9-119DEF43FB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1F5DD2F-2639-40BA-AD12-ACE999E5F1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="2280" windowWidth="15375" windowHeight="7785" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Faltantes febrero" sheetId="5" state="hidden" r:id="rId1"/>
@@ -61207,26 +61207,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2c384499-6772-4313-ae8f-2d1143638ba0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c5be7662-c91c-4034-9f32-6ea20118eb9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E037D65041E8ED4584DA28C16A4927B6" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e4ccadbacc0716b3b5321683b5360436">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2c384499-6772-4313-ae8f-2d1143638ba0" xmlns:ns3="c5be7662-c91c-4034-9f32-6ea20118eb9e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="125bb9dac04b723b6d4bd9d405926887" ns2:_="" ns3:_="">
     <xsd:import namespace="2c384499-6772-4313-ae8f-2d1143638ba0"/>
@@ -61467,26 +61447,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5756C0BD-24D8-4C86-9FB1-3653DB3EE7D6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2c384499-6772-4313-ae8f-2d1143638ba0"/>
-    <ds:schemaRef ds:uri="c5be7662-c91c-4034-9f32-6ea20118eb9e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA678AD8-784E-46F3-8189-78ED809039A7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2c384499-6772-4313-ae8f-2d1143638ba0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c5be7662-c91c-4034-9f32-6ea20118eb9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC7E1C22-4BCD-4768-BF4C-C5E2A8AC6698}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -61503,4 +61484,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA678AD8-784E-46F3-8189-78ED809039A7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5756C0BD-24D8-4C86-9FB1-3653DB3EE7D6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2c384499-6772-4313-ae8f-2d1143638ba0"/>
+    <ds:schemaRef ds:uri="c5be7662-c91c-4034-9f32-6ea20118eb9e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>